<commit_message>
Fix duplicate records in all datasets
State scraper: deduplicate by transaction URL during scrape
FEC scraper: added transaction_id field, deduplicate during scrape
Deduped existing data files:
- State 2026: 88,479 -> 56,073 rows (37% were dupes)
- Federal 2026 receipts: 83,489 -> 48,170 (42%)
- Federal 2024 receipts: 32,659 -> 25,952 (21%)
- Federal expenditures: minor dedup (2-3%)
Re-ran R aggregation with clean data
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -484,7 +484,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1351701.29</v>
+        <v>833728.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1232143.5</v>
+        <v>726111.79</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -520,7 +520,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>jonathan bush</t>
+          <t>angus s king iii</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -530,11 +530,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>926861</v>
+        <v>577821.36</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>angus s king iii</t>
+          <t>jonathan bush</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -555,11 +555,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
-        <v>858719.6899999999</v>
+        <v>538616</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -584,7 +584,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>724500.6800000001</v>
+        <v>445549.88</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>641479.13</v>
+        <v>374519.88</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>490095</v>
+        <v>327070</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>392786.08</v>
+        <v>271405.58</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>332962</v>
+        <v>239331</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>289540.83</v>
+        <v>201197.62</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>269275</v>
+        <v>180548</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>27630.46</v>
+        <v>16677.67</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
         </is>
       </c>
       <c r="E16">
-        <v>665</v>
+        <v>645</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>275</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2620</v>
+        <v>2560</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1682,7 +1682,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1710,7 +1710,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1780,7 +1780,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5900</v>
+        <v>2800</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2018,7 +2018,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2116,7 +2116,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>946.0799999999999</v>
+        <v>550.54</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>170</v>
+        <v>110</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2494,7 +2494,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>23460</v>
+        <v>17705</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2522,7 +2522,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>675</v>
+        <v>575</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2690,7 +2690,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>720</v>
+        <v>420</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2984,7 +2984,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>395</v>
+        <v>260</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>833</v>
+        <v>504</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3222,7 +3222,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3460,7 +3460,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>974.49</v>
+        <v>640.26</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3530,7 +3530,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>816.64</v>
+        <v>408.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3600,7 +3600,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>950</v>
+        <v>475</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3894,7 +3894,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1001.22</v>
+        <v>751.22</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3964,7 +3964,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4174,7 +4174,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4272,7 +4272,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4440,20 +4440,90 @@
         </is>
       </c>
       <c r="E3">
+        <v>500</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_106</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>trevor alex doiron</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>76</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
         <v>1000</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Representative_106</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_76</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4493,16 +4563,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>trevor alex doiron</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>76</v>
+          <t>woodleigh h hughes</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>78</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -4510,20 +4580,90 @@
         </is>
       </c>
       <c r="E2">
+        <v>700</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_78</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>christopher alfred lewey</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>82</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
         <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Representative_76</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>Representative_82</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4563,37 +4703,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>woodleigh h hughes</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>78</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>700</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Representative_78</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>kimberly j pomerleau</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>85</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>790</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_85</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4633,37 +4773,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>christopher alfred lewey</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>82</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>1000</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Representative_82</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>david wayne boyer jr</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>87</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>3483.7</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_87</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -4703,16 +4843,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>kimberly j pomerleau</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>85</v>
+          <t>laurel libby</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>90</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -4720,147 +4860,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1110</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Representative_85</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>david wayne boyer jr</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>87</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Republican</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>4408.7</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Representative_87</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>laurel libby</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>90</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Republican</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>79297.60000000001</v>
+        <v>56333.3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7140</v>
+        <v>6065</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4986,7 +4986,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>4751.73</v>
+        <v>2628.64</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5196,7 +5196,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1300</v>
+        <v>1100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3575</v>
+        <v>3325</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5406,7 +5406,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>950</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5714,7 +5714,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>800</v>
+        <v>400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5784,20 +5784,300 @@
         </is>
       </c>
       <c r="E2">
+        <v>50</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_21</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>nathan burnett</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>22</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>1789.2</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_22</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>matthea elisabeth larsen daughtry</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>23</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>20</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_23</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>denise tepler</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>24</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>225</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_24</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>april fournier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>114</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
         <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Senator_21</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet67.xml><?xml version="1.0" encoding="utf-8"?>
+          <t>Representative_114</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -5837,7 +6117,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nathan burnett</t>
+          <t>teresa s pierce</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5846,7 +6126,7 @@
         </is>
       </c>
       <c r="C2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -5854,20 +6134,20 @@
         </is>
       </c>
       <c r="E2">
-        <v>1789.2</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senator_22</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet68.xml><?xml version="1.0" encoding="utf-8"?>
+        <v>2400</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_25</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -5907,7 +6187,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>matthea elisabeth larsen daughtry</t>
+          <t>peter g violette</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5916,286 +6196,6 @@
         </is>
       </c>
       <c r="C2">
-        <v>23</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>20</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senator_23</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet69.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>denise tepler</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Senator</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>24</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>225</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senator_24</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>april fournier</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>114</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>200</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Representative_114</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet70.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>teresa s pierce</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Senator</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>25</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>2400</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senator_25</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet71.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>peter g violette</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Senator</t>
-        </is>
-      </c>
-      <c r="C2">
         <v>26</v>
       </c>
       <c r="D2" t="inlineStr">
@@ -6204,7 +6204,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>2600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6372,7 +6372,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9645.309999999999</v>
+        <v>8295.309999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2750</v>
+        <v>2250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6470,7 +6470,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1420</v>
+        <v>1110</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6596,7 +6596,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6694,7 +6694,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2257</v>
+        <v>1661</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6764,7 +6764,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3750</v>
+        <v>2600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2225</v>
+        <v>1725</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6890,7 +6890,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1390</v>
+        <v>1290</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>570</v>
+        <v>335</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7086,7 +7086,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1250</v>
+        <v>750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7366,7 +7366,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update state data through April 30, export Senate race spreadsheets, regenerate clean data
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -4778,7 +4778,7 @@
 
 <file path=xl/worksheets/sheet137.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4838,82 +4838,110 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>Senator_7</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>candidate</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>race</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>district</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>party</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>tot_con_per_cand</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sheet_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>michael tipping</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Senator</t>
-        </is>
-      </c>
-      <c r="C2">
-        <v>8</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E2">
-        <v>3050</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Senator_8</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>cheryl hewes</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>7</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>35.71</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_7</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet138.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>race</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>district</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>party</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>tot_con_per_cand</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sheet_name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>michael tipping</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E2">
+        <v>3050</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Senator_8</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>leo christopher kenney</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add Zachary Lejonhud and Azalea Cormier, regenerate data
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -4165,7 +4165,7 @@
 
 <file path=xl/worksheets/sheet118.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4203,7 +4203,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>amanda noelle collamore</t>
+          <t>zachary lejonhud</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4214,13 +4214,8 @@
       <c r="C2">
         <v>68</v>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Republican</t>
-        </is>
-      </c>
       <c r="E2">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4231,7 +4226,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>brian j blake</t>
+          <t>amanda noelle collamore</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4244,13 +4239,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_68</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>brian j blake</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>68</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_68</t>
         </is>
@@ -6428,7 +6451,7 @@
 
 <file path=xl/worksheets/sheet132.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -6522,7 +6545,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>caldwell jackson</t>
+          <t>azalea cormier</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6533,13 +6556,8 @@
       <c r="C4">
         <v>80</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Republican</t>
-        </is>
-      </c>
       <c r="E4">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -6550,7 +6568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>roberta j hill</t>
+          <t>caldwell jackson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -6563,13 +6581,41 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>Representative_80</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>roberta j hill</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>80</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Representative_80</t>
         </is>

</xml_diff>

<commit_message>
Exclude special election transactions from main analysis — fixes Harriman $33K -> $250
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -8820,7 +8820,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>33315.76</v>
+        <v>250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8831,7 +8831,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>janet beaudoin</t>
+          <t>kendil elizabeth snowblack</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8848,7 +8848,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>13041</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8859,7 +8859,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kendil elizabeth snowblack</t>
+          <t>kristen sarah cloutier</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8872,7 +8872,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
@@ -8887,7 +8887,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>kristen sarah cloutier</t>
+          <t>janet beaudoin</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8900,7 +8900,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">

</xml_diff>

<commit_message>
Fresh scrape: 128,737 rows, exact match with site, 0 duplicates, name merges fixed
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -1125,7 +1125,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>angus s iii king</t>
+          <t>angus king iii</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3979,7 +3979,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>michael perkins</t>
+          <t>michael d perkins</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9167,7 +9167,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>joseph edwards velozo</t>
+          <t>luke jensen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9178,13 +9178,8 @@
       <c r="C4">
         <v>96</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Republican</t>
-        </is>
-      </c>
       <c r="E4">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9195,7 +9190,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>david c projansky</t>
+          <t>joseph edwards velozo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -9208,7 +9203,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
@@ -9223,7 +9218,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>luke dylan jensen</t>
+          <t>david c projansky</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9233,6 +9228,11 @@
       </c>
       <c r="C6">
         <v>96</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
       </c>
       <c r="E6">
         <v>0</v>
@@ -12800,7 +12800,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2855</v>
+        <v>2850</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18051,7 +18051,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>michael cunningham ii</t>
+          <t>michael hobart cunningham ii</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -20001,7 +20001,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>rebecca flood andrews</t>
+          <t>rebecca lynn flood andrews</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -23533,7 +23533,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>anthony weaver</t>
+          <t>anthony m weaver</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -26649,7 +26649,7 @@
 
 <file path=xl/worksheets/sheet91.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -26827,7 +26827,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>christopher austin</t>
+          <t>ann h matlack</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -26840,41 +26840,13 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
-        <is>
-          <t>Representative_43</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ann h matlack</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Representative</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>43</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Democratic</t>
-        </is>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr">
         <is>
           <t>Representative_43</t>
         </is>
@@ -27587,7 +27559,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>james william iii hunt</t>
+          <t>erik hobson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -27604,7 +27576,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -27615,7 +27587,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>holly beth stover</t>
+          <t>james william iii hunt</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -27628,7 +27600,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E4">
@@ -27643,7 +27615,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>erik hobson</t>
+          <t>holly beth stover</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -27656,7 +27628,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E5">

</xml_diff>

<commit_message>
Add Jack McCarthy (Rep 3, TF) — new candidate just added to disclosure site today
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -16930,7 +16930,7 @@
 
 <file path=xl/worksheets/sheet76.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -17016,6 +17016,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jack mccarthy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_3</t>
         </is>

</xml_diff>

<commit_message>
Move Cherry to H38, add Goble to H18, remove from Governor
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -537,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -975,7 +975,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>jason cherry</t>
+          <t>john michael glowa sr</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -985,11 +985,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E18">
-        <v>310</v>
+        <v>180</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>john michael glowa sr</t>
+          <t>andrew parker</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1014,34 +1014,9 @@
         </is>
       </c>
       <c r="E19">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="F19" t="inlineStr">
-        <is>
-          <t>Governor</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>andrew parker</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Governor</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Unenrolled</t>
-        </is>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20" t="inlineStr">
         <is>
           <t>Governor</t>
         </is>
@@ -15502,7 +15477,7 @@
 
 <file path=xl/worksheets/sheet63.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -15560,6 +15535,34 @@
         <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_18</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jonathan goble</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>18</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>880.54</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Representative_18</t>
         </is>
@@ -17910,7 +17913,7 @@
 
 <file path=xl/worksheets/sheet85.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -17948,7 +17951,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>benjamin charles hymes</t>
+          <t>jason cherry</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17961,11 +17964,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>310</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17976,7 +17979,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kayla miller</t>
+          <t>benjamin charles hymes</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17989,13 +17992,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_38</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>kayla miller</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>38</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_38</t>
         </is>

</xml_diff>

<commit_message>
Add H29 special election section — two races on one page
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -16779,7 +16779,7 @@
 
 <file path=xl/worksheets/sheet75.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -16845,7 +16845,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>james michael michaud</t>
+          <t>nancy theriaultspecial</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16873,7 +16873,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nancy jean theriault</t>
+          <t>james michael michaud</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16901,7 +16901,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nancy mcdowell</t>
+          <t>nancy jean theriault</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16914,13 +16914,41 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
+        <is>
+          <t>Representative_29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nancy mcdowell</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>29</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>Representative_29</t>
         </is>

</xml_diff>

<commit_message>
Apply colleague's audit: display names, add/unhide candidates, dropped out labels
- 10 display name fixes (Glowa, Kalloch, Mitchell, Litalien, Carlisle, Contreni, Bridges, Olsen, Winslow, Runte)
- Add: James Libby (Gov, dropped out), Lawrence Bessey (H58), Bret Martel (H95), Lauren Jones (H112)
- Unhide + label dropped out: Louis Larios (H51), Nicole Bambrick (H77), Lisa Nelthropp (H113)
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -537,7 +537,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -975,7 +975,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>john michael glowa sr</t>
+          <t>james libby</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -985,11 +985,11 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E18">
-        <v>180</v>
+        <v>364.7</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1000,23 +1000,48 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>john michael glowa sr</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Governor</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E19">
+        <v>180</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Governor</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>andrew parker</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Governor</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Unenrolled</t>
         </is>
       </c>
-      <c r="E19">
+      <c r="E20">
         <v>0</v>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Governor</t>
         </is>
@@ -1127,7 +1152,7 @@
 
 <file path=xl/worksheets/sheet100.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1213,6 +1238,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_51</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>louis larios</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>51</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_51</t>
         </is>
@@ -1841,7 +1894,7 @@
 
 <file path=xl/worksheets/sheet107.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1955,6 +2008,34 @@
         <v>755</v>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>Representative_58</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>lawrence e bessey jr</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>58</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Representative_58</t>
         </is>
@@ -4207,7 +4288,7 @@
 
 <file path=xl/worksheets/sheet128.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -4293,6 +4374,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_77</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>nicole bambrick</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>77</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_77</t>
         </is>
@@ -6419,7 +6528,7 @@
 
 <file path=xl/worksheets/sheet148.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -6485,7 +6594,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>matthew kershaw</t>
+          <t>bret michael martel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6498,13 +6607,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_95</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>matthew kershaw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>95</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_95</t>
         </is>
@@ -8799,7 +8936,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -8857,6 +8994,34 @@
         <v>3325</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_112</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lauren chelsea jones</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>112</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Representative_112</t>
         </is>
@@ -9849,7 +10014,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -9907,6 +10072,34 @@
         <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_113</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lisa nelthropp</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>113</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Representative_113</t>
         </is>

</xml_diff>

<commit_message>
Update site with deduped state data — fix inflated candidate totals
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2190265.3</v>
+        <v>1892270.95</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1877877.51</v>
+        <v>1673857.13</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1520770</v>
+        <v>1406495</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nirav shah</t>
+          <t>angus s king iii</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>1406661.85</v>
+        <v>1171439.47</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>angus s king iii</t>
+          <t>nirav shah</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1261086.74</v>
+        <v>1149771.54</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>troy dale jackson</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -710,11 +710,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E7">
-        <v>1035139.12</v>
+        <v>841282.88</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>troy dale jackson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -735,11 +735,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E8">
-        <v>906579.88</v>
+        <v>828772.21</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>699659.96</v>
+        <v>626612.97</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>510482.78</v>
+        <v>456282.78</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>389224</v>
+        <v>362524</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>359773</v>
+        <v>224521</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>191285.43</v>
+        <v>160788.38</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>44809.14</v>
+        <v>40266.84</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E17">
-        <v>1390</v>
+        <v>1290</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3650</v>
+        <v>1800</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3750</v>
+        <v>2400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1360</v>
+        <v>1310</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8328.210000000001</v>
+        <v>7619.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3130</v>
+        <v>2860</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2600</v>
+        <v>1050</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9450</v>
+        <v>6550</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2585</v>
+        <v>2230</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1656</v>
+        <v>1256</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3209,7 +3209,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1162</v>
+        <v>606</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1920</v>
+        <v>1870</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1526.15</v>
+        <v>966.15</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1400</v>
+        <v>900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8345</v>
+        <v>5685</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5075</v>
+        <v>3225</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1800</v>
+        <v>900</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>610</v>
+        <v>305</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>14355</v>
+        <v>12255</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2250</v>
+        <v>2150</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2600</v>
+        <v>1100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5887.6</v>
+        <v>5512.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>760</v>
+        <v>380</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4844,7 +4844,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>azalea cormier</t>
+          <t>gino valeriani</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4857,11 +4857,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1315</v>
+        <v>830</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4872,7 +4872,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gino valeriani</t>
+          <t>azalea cormier</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4885,11 +4885,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
-        <v>830</v>
+        <v>665</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1300</v>
+        <v>650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2283.65</v>
+        <v>1883.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2033.78</v>
+        <v>1736.89</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5771,7 +5771,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6383.4</v>
+        <v>2591.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13436.25</v>
+        <v>11226.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>90627.3</v>
+        <v>80627.3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1200</v>
+        <v>700</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8723.02</v>
+        <v>7172.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>528.02</v>
+        <v>264.01</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>135</v>
+        <v>85</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>262</v>
+        <v>131</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7255,7 +7255,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7717,7 +7717,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7843,7 +7843,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1490</v>
+        <v>1390</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8011,7 +8011,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>450</v>
+        <v>275</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2225.5</v>
+        <v>1225.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9104.48</v>
+        <v>7604.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2965</v>
+        <v>2915</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8288,7 +8288,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>joseph edward martin</t>
+          <t>peter j southam</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8301,11 +8301,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>3100</v>
+        <v>2835</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>peter j southam</t>
+          <t>joseph edward martin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8329,11 +8329,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>2835</v>
+        <v>1100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8599,7 +8599,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17885</v>
+        <v>15355</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3108</v>
+        <v>2988</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>695</v>
+        <v>395</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8921,7 +8921,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5150</v>
+        <v>4650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3825</v>
+        <v>3575</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9089,7 +9089,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3500</v>
+        <v>3400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1840</v>
+        <v>1740</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>33000</v>
+        <v>17000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9453,7 +9453,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>12855</v>
+        <v>7830</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9523,7 +9523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11132.51</v>
+        <v>10932.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9971,7 +9971,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6590</v>
+        <v>4490</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10150,7 +10150,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>daniel sayre</t>
+          <t>jonathan reed fallon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>3055</v>
+        <v>3044</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10178,7 +10178,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jonathan reed fallon</t>
+          <t>daniel sayre</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10191,11 +10191,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>3044</v>
+        <v>2930</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10265,7 +10265,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6002</v>
+        <v>6001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10391,7 +10391,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6225</v>
+        <v>5725</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10419,7 +10419,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5518.7</v>
+        <v>4539</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10447,7 +10447,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>5050</v>
+        <v>4050</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10671,7 +10671,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13170</v>
+        <v>11865</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1440</v>
+        <v>720</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>642</v>
+        <v>446</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11161,7 +11161,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>34063.6</v>
+        <v>16643.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11259,7 +11259,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4900</v>
+        <v>3315</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>277</v>
+        <v>227</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11637,7 +11637,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>900</v>
+        <v>600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>40165</v>
+        <v>28216</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12099,7 +12099,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5250</v>
+        <v>3250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12659,7 +12659,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12757,7 +12757,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13191,7 +13191,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3270</v>
+        <v>3120</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13583,7 +13583,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3325</v>
+        <v>1775</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13681,7 +13681,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13779,7 +13779,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3310</v>
+        <v>2305</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13877,7 +13877,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5600</v>
+        <v>4600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13975,7 +13975,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7620</v>
+        <v>3145</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14129,7 +14129,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>350</v>
+        <v>175</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14423,7 +14423,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14966,7 +14966,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>timothy towne</t>
+          <t>mallory aaren cook</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14979,11 +14979,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14994,7 +14994,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>mallory aaren cook</t>
+          <t>timothy towne</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15007,11 +15007,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15305,7 +15305,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1990</v>
+        <v>1350</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15753,7 +15753,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>950.54</v>
+        <v>915.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16145,7 +16145,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>325</v>
+        <v>225</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16425,7 +16425,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>395</v>
+        <v>295</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -16635,7 +16635,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2012</v>
+        <v>1691</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16831,7 +16831,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>820</v>
+        <v>810</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16859,7 +16859,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>210</v>
+        <v>110</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17209,7 +17209,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5900</v>
+        <v>2950</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>495</v>
+        <v>480</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17601,7 +17601,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>14931.76</v>
+        <v>11781.76</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17699,7 +17699,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2200</v>
+        <v>1600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17797,7 +17797,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2250</v>
+        <v>1250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18217,7 +18217,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18903,7 +18903,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5681.8</v>
+        <v>5156.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18931,7 +18931,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3100</v>
+        <v>2470</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19057,7 +19057,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5769.8</v>
+        <v>3919.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1570.65</v>
+        <v>1370.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19113,7 +19113,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1127.68</v>
+        <v>563.84</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19183,7 +19183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16565</v>
+        <v>14715</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19211,7 +19211,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>4093.18</v>
+        <v>3455.68</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Revert dedup — need to verify against site before removing any transactions
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1892270.95</v>
+        <v>2190265.3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1673857.13</v>
+        <v>1877877.51</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1406495</v>
+        <v>1520770</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>angus s king iii</t>
+          <t>nirav shah</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>1171439.47</v>
+        <v>1406661.85</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nirav shah</t>
+          <t>angus s king iii</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1149771.54</v>
+        <v>1261086.74</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>troy dale jackson</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -710,11 +710,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E7">
-        <v>841282.88</v>
+        <v>1035139.12</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>troy dale jackson</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -735,11 +735,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E8">
-        <v>828772.21</v>
+        <v>906579.88</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>626612.97</v>
+        <v>699659.96</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>456282.78</v>
+        <v>510482.78</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>362524</v>
+        <v>389224</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>224521</v>
+        <v>359773</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>160788.38</v>
+        <v>191285.43</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>40266.84</v>
+        <v>44809.14</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E17">
-        <v>1290</v>
+        <v>1390</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1800</v>
+        <v>3650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2400</v>
+        <v>3750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1310</v>
+        <v>1360</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7619.56</v>
+        <v>8328.210000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2860</v>
+        <v>3130</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>2600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6550</v>
+        <v>9450</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2230</v>
+        <v>2585</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1256</v>
+        <v>1656</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3209,7 +3209,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>606</v>
+        <v>1162</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1870</v>
+        <v>1920</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3531,7 +3531,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>966.15</v>
+        <v>1526.15</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3601,7 +3601,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>900</v>
+        <v>1400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5685</v>
+        <v>8345</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3225</v>
+        <v>5075</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>900</v>
+        <v>1800</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>305</v>
+        <v>610</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12255</v>
+        <v>14355</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4147,7 +4147,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2150</v>
+        <v>2250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4343,7 +4343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1100</v>
+        <v>2600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5512.6</v>
+        <v>5887.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4595,7 +4595,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>380</v>
+        <v>760</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4693,7 +4693,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4844,7 +4844,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gino valeriani</t>
+          <t>azalea cormier</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4857,11 +4857,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>830</v>
+        <v>1315</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4872,7 +4872,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>azalea cormier</t>
+          <t>gino valeriani</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4885,11 +4885,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E4">
-        <v>665</v>
+        <v>830</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>650</v>
+        <v>1300</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1883.65</v>
+        <v>2283.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5379,7 +5379,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>800</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1736.89</v>
+        <v>2033.78</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5771,7 +5771,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2591.7</v>
+        <v>6383.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5869,7 +5869,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11226.25</v>
+        <v>13436.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6065,7 +6065,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>80627.3</v>
+        <v>90627.3</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>700</v>
+        <v>1200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7172.02</v>
+        <v>8723.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6611,7 +6611,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>264.01</v>
+        <v>528.02</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6737,7 +6737,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>85</v>
+        <v>135</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6807,7 +6807,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7157,7 +7157,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>131</v>
+        <v>262</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7255,7 +7255,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7717,7 +7717,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7843,7 +7843,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1390</v>
+        <v>1490</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8011,7 +8011,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>275</v>
+        <v>450</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8081,7 +8081,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1225.5</v>
+        <v>2225.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8207,7 +8207,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7604.48</v>
+        <v>9104.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2915</v>
+        <v>2965</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8288,7 +8288,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>peter j southam</t>
+          <t>joseph edward martin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8301,11 +8301,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>2835</v>
+        <v>3100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8316,7 +8316,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>joseph edward martin</t>
+          <t>peter j southam</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8329,11 +8329,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>1100</v>
+        <v>2835</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8599,7 +8599,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15355</v>
+        <v>17885</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8627,7 +8627,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2988</v>
+        <v>3108</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8851,7 +8851,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>395</v>
+        <v>695</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8921,7 +8921,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4650</v>
+        <v>5150</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3575</v>
+        <v>3825</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9089,7 +9089,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3400</v>
+        <v>3500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9285,7 +9285,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1740</v>
+        <v>1840</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9425,7 +9425,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17000</v>
+        <v>33000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9453,7 +9453,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>7830</v>
+        <v>12855</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9523,7 +9523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>10932.51</v>
+        <v>11132.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9971,7 +9971,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4490</v>
+        <v>6590</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10150,7 +10150,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jonathan reed fallon</t>
+          <t>daniel sayre</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10163,11 +10163,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>3044</v>
+        <v>3055</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10178,7 +10178,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>daniel sayre</t>
+          <t>jonathan reed fallon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10191,11 +10191,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>2930</v>
+        <v>3044</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10265,7 +10265,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6001</v>
+        <v>6002</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10391,7 +10391,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5725</v>
+        <v>6225</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10419,7 +10419,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>4539</v>
+        <v>5518.7</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10447,7 +10447,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>4050</v>
+        <v>5050</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10671,7 +10671,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11865</v>
+        <v>13170</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11021,7 +11021,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>720</v>
+        <v>1440</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>446</v>
+        <v>642</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11161,7 +11161,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16643.8</v>
+        <v>34063.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11259,7 +11259,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3315</v>
+        <v>4900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>227</v>
+        <v>277</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11637,7 +11637,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11735,7 +11735,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>28216</v>
+        <v>40165</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12099,7 +12099,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3250</v>
+        <v>5250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12659,7 +12659,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>195</v>
+        <v>230</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12757,7 +12757,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13191,7 +13191,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3120</v>
+        <v>3270</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13583,7 +13583,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1775</v>
+        <v>3325</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13681,7 +13681,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>4000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13779,7 +13779,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2305</v>
+        <v>3310</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13877,7 +13877,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4600</v>
+        <v>5600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13975,7 +13975,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3145</v>
+        <v>7620</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14129,7 +14129,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>175</v>
+        <v>350</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -14325,7 +14325,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14423,7 +14423,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14966,7 +14966,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mallory aaren cook</t>
+          <t>timothy towne</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14979,11 +14979,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14994,7 +14994,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>timothy towne</t>
+          <t>mallory aaren cook</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15007,11 +15007,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -15109,7 +15109,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15305,7 +15305,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1350</v>
+        <v>1990</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15753,7 +15753,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>915.54</v>
+        <v>950.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16145,7 +16145,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>225</v>
+        <v>325</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16425,7 +16425,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>295</v>
+        <v>395</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -16635,7 +16635,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1691</v>
+        <v>2012</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16831,7 +16831,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>810</v>
+        <v>820</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16859,7 +16859,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>110</v>
+        <v>210</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17209,7 +17209,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2950</v>
+        <v>5900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17601,7 +17601,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11781.76</v>
+        <v>14931.76</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17699,7 +17699,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>2200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17797,7 +17797,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1250</v>
+        <v>2250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18217,7 +18217,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18903,7 +18903,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5156.8</v>
+        <v>5681.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18931,7 +18931,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2470</v>
+        <v>3100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19057,7 +19057,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3919.8</v>
+        <v>5769.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19085,7 +19085,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1370.65</v>
+        <v>1570.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19113,7 +19113,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>563.84</v>
+        <v>1127.68</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19183,7 +19183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>14715</v>
+        <v>16565</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19211,7 +19211,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3455.68</v>
+        <v>4093.18</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix McDowell regular: replace with 14 site-verified transactions
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -17038,7 +17038,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nancy theriaultspecial</t>
+          <t>nancy mcdowell</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17051,11 +17051,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>925</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17066,7 +17066,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>james michael michaud</t>
+          <t>nancy theriaultspecial</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17094,7 +17094,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nancy jean theriault</t>
+          <t>james michael michaud</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17122,7 +17122,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nancy mcdowell</t>
+          <t>nancy jean theriault</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -17135,7 +17135,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E6">

</xml_diff>

<commit_message>
Fix Nancy Theriault: replace with 16 site-verified transactions
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -17066,7 +17066,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nancy theriaultspecial</t>
+          <t>nancy jean theriault</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17083,7 +17083,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>525</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17094,7 +17094,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>james michael michaud</t>
+          <t>nancy theriaultspecial</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17122,7 +17122,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nancy jean theriault</t>
+          <t>james michael michaud</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>

<commit_message>
Fix name matching: add 72 name merges, apply to transactions in R script
Fixes $108K in missing expenditures and $140K in missing contributions
caused by filer name variants (middle names, suffixes, punctuation)
not matching candidate list entries.
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -900,7 +900,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>w edward crockett</t>
+          <t>james libby</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -910,11 +910,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E15">
-        <v>8835</v>
+        <v>15259.7</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>kenneth a capron</t>
+          <t>w edward crockett</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -935,11 +935,11 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E16">
-        <v>3450</v>
+        <v>8835</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>derek allen levasseur</t>
+          <t>kenneth a capron</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -960,11 +960,11 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E17">
-        <v>1150</v>
+        <v>3450</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>john michael glowa sr</t>
+          <t>derek allen levasseur</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1000,7 +1000,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>james libby</t>
+          <t>john michael glowa sr</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1010,11 +1010,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E19">
-        <v>364.7</v>
+        <v>1150</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>david wayne guilmette</t>
+          <t>sally jeane cluchey</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1329,11 +1329,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>820</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1344,7 +1344,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sally jeane cluchey</t>
+          <t>david wayne guilmette</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1357,11 +1357,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>820</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1414,7 +1414,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>richard marc goldman</t>
+          <t>michael h lemelin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1427,11 +1427,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1442,7 +1442,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>michael h lemelin</t>
+          <t>richard marc goldman</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1455,11 +1455,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2506,7 +2506,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>robin crawley</t>
+          <t>alicia c collins</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>202</v>
+        <v>9175.120000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2534,7 +2534,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>alicia c collins</t>
+          <t>robin crawley</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2547,11 +2547,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>202</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>523</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3307,7 +3307,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3433,7 +3433,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4200,7 +4200,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>trevor alex doiron</t>
+          <t>sheila a lyman</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4213,7 +4213,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
@@ -4228,7 +4228,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>clinton brooks</t>
+          <t>trevor alex doiron</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4241,11 +4241,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4256,7 +4256,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>sheila a lyman</t>
+          <t>clinton brooks</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
@@ -4763,7 +4763,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>700</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1200</v>
+        <v>1201.53</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1170</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6468,7 +6468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>scott a harriman</t>
+          <t>janet beaudoin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6481,11 +6481,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6496,7 +6496,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>janet beaudoin</t>
+          <t>scott a harriman</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6509,11 +6509,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6790,7 +6790,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>jason lewis copp</t>
+          <t>christina rue cork mitchell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
@@ -6818,7 +6818,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>christina rue cork mitchell</t>
+          <t>jason lewis copp</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6831,11 +6831,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7059,7 +7059,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -7210,7 +7210,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vaughn j mclaughlin</t>
+          <t>lucien daigle</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7223,11 +7223,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1634</v>
+        <v>2555</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7238,7 +7238,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lucien daigle</t>
+          <t>vaughn j mclaughlin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7251,11 +7251,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>155</v>
+        <v>1634</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7700,7 +7700,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>steven mcgee</t>
+          <t>craig v hickman</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7713,11 +7713,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>3500</v>
+        <v>4400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7728,7 +7728,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>craig v hickman</t>
+          <t>steven mcgee</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7741,11 +7741,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>3500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9142,7 +9142,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>peter g violette</t>
+          <t>kenneth james cianchette</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9159,7 +9159,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3000</v>
+        <v>9450</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9170,7 +9170,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>timothy e nangle</t>
+          <t>peter g violette</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9183,11 +9183,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>2975</v>
+        <v>3000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9198,7 +9198,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kenneth james cianchette</t>
+          <t>timothy e nangle</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9211,11 +9211,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2975</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10069,7 +10069,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10682,7 +10682,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>aaron dana</t>
+          <t>kenneth davis jr</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10695,11 +10695,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>925</v>
+        <v>3000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10710,7 +10710,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kenneth davis jr</t>
+          <t>aaron dana</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -10723,11 +10723,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>925</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -12449,7 +12449,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>2100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12810,7 +12810,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>todd michael davis</t>
+          <t>lynn holland copeland</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -12823,11 +12823,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12838,7 +12838,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>lynn holland copeland</t>
+          <t>todd michael davis</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12851,11 +12851,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13023,7 +13023,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13289,7 +13289,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>275</v>
+        <v>1275</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13468,7 +13468,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>michelle kathryn conners</t>
+          <t>john michael eder</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -13481,11 +13481,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>2500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13496,7 +13496,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>john michael eder</t>
+          <t>michelle kathryn conners</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -14700,7 +14700,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>walter gerard jr runte</t>
+          <t>bradley s moulton</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14713,11 +14713,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14728,7 +14728,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bradley s moulton</t>
+          <t>walter gerard jr runte</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -15403,7 +15403,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15627,7 +15627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>13010</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16243,7 +16243,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17797,7 +17797,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2250</v>
+        <v>3500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18074,7 +18074,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>alan lee orcutt</t>
+          <t>reagan leeann paul</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18087,11 +18087,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>950</v>
+        <v>15250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18102,7 +18102,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>reagan leeann paul</t>
+          <t>alan lee orcutt</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18115,11 +18115,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>950</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18245,7 +18245,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -18466,7 +18466,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d michael ray</t>
+          <t>joseph milton mclaughlin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18479,11 +18479,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1150</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18494,7 +18494,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>joseph milton mclaughlin</t>
+          <t>d michael ray</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18507,11 +18507,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18707,7 +18707,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Apply George's editorial updates: 46 not-on-ballot, 6 new independents, name/party changes
- 46 candidates labeled (not on ballot) including James Libby
- Billy Faulkingham renamed to Billy Bob Faulkingham
- Eric Small: Republican to Unenrolled/independent
- 6 new independent candidates added (Duguay, Gott, Shaw, McWilliams, Lessard, Cobb)
- Roy Gott tagged MCEA
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -7466,7 +7466,7 @@
 
 <file path=xl/worksheets/sheet156.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -7552,6 +7552,34 @@
         <v>200</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>roy gott</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>12</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Senator_12</t>
         </is>
@@ -8250,7 +8278,7 @@
 
 <file path=xl/worksheets/sheet163.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -8336,6 +8364,34 @@
         <v>2835</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_19</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>david duguay</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>19</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Senator_19</t>
         </is>
@@ -12534,7 +12590,7 @@
 
 <file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -12592,6 +12648,34 @@
         <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_128</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>lawrence mcwilliams</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>128</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Representative_128</t>
         </is>
@@ -13136,7 +13220,7 @@
 
 <file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -13194,6 +13278,34 @@
         <v>3100</v>
       </c>
       <c r="F2" t="inlineStr">
+        <is>
+          <t>Representative_133</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>marc lessard</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>133</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Representative_133</t>
         </is>
@@ -14419,7 +14531,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E2">
@@ -14830,7 +14942,7 @@
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14916,6 +15028,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_148</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>noah cobb</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>148</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_148</t>
         </is>
@@ -16678,7 +16818,7 @@
 
 <file path=xl/worksheets/sheet72.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -16764,6 +16904,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>adam shaw</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>26</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_26</t>
         </is>

</xml_diff>

<commit_message>
Weekly update July 14: 372 new state transactions, fresh FEC totals
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1250</v>
+        <v>1370</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>21.15</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4665,7 +4665,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>250</v>
+        <v>750</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5351,7 +5351,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2072.9</v>
+        <v>2213.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1896.89</v>
+        <v>2721.89</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14185,7 +14185,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1672.72</v>
+        <v>2472.72</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14531,7 +14531,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
@@ -14997,7 +14997,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16537,7 +16537,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>760</v>
+        <v>792.27</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17584,7 +17584,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>andrew r torbett</t>
+          <t>eric boothroyd</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17597,11 +17597,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>510</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17612,7 +17612,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>eric boothroyd</t>
+          <t>andrew r torbett</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17625,11 +17625,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19225,7 +19225,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4769.8</v>
+        <v>8019.8</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly update July 22: Roberts Q2, Cobb dropout, 56K new Q2 itemized receipts from raw filings
- Roberts Q2 filing: COH $4,893, disbursements $15,158
- Noah Cobb (House 148) marked as dropped out
- Parsed 17 raw FEC filing files to fill Q2 Schedule A/B gaps (56K receipts, 1.5K expenditures)
- Fixed contributor/payee name case normalization in R script
- Fixed earmarked-conduit double-counting in platform totals
- State scraper: 160K rows (+8K new transactions through July 7)
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2050515.93</v>
+        <v>2432116.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1663628.1</v>
+        <v>1672883.28</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>1244866.65</v>
+        <v>1246868.85</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1193608.86</v>
+        <v>1194028.86</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>907375.0699999999</v>
+        <v>912130.76</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>725903.62</v>
+        <v>778029.76</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>656791.97</v>
+        <v>688181.97</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>386123</v>
+        <v>386477.21</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>337068</v>
+        <v>337118</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>44598.19</v>
+        <v>44638.19</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2700</v>
+        <v>3300</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>202</v>
+        <v>211</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4500</v>
+        <v>4700</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3503,7 +3503,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2020</v>
+        <v>2070</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3895,7 +3895,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3925</v>
+        <v>4425</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4119,7 +4119,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13970</v>
+        <v>15070</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4469,7 +4469,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>2350</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5925</v>
+        <v>6025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4763,7 +4763,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>700</v>
+        <v>1200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1500</v>
+        <v>2200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5138,7 +5138,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>timothy becker</t>
+          <t>marygrace caroline cimino</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5151,11 +5151,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>2080</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5166,7 +5166,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>marygrace caroline cimino</t>
+          <t>timothy becker</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5179,11 +5179,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>650</v>
+        <v>675</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>300</v>
+        <v>612</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5477,7 +5477,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2721.89</v>
+        <v>2821.89</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5575,7 +5575,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6183.7</v>
+        <v>6783.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6485,7 +6485,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>3850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6790,7 +6790,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>christina rue cork mitchell</t>
+          <t>jason lewis copp</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6803,11 +6803,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6818,7 +6818,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jason lewis copp</t>
+          <t>christina rue cork mitchell</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6831,7 +6831,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -7728,7 +7728,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>craig v hickman</t>
+          <t>steven mcgee</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7741,11 +7741,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>4400</v>
+        <v>5000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7756,7 +7756,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>steven mcgee</t>
+          <t>craig v hickman</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7769,11 +7769,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>3500</v>
+        <v>4733.34</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8655,7 +8655,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>18280</v>
+        <v>19730</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8977,7 +8977,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4425</v>
+        <v>5775</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9047,7 +9047,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3575</v>
+        <v>4075</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9215,7 +9215,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9450</v>
+        <v>12000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9579,7 +9579,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11406.51</v>
+        <v>12406.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5925</v>
+        <v>6425</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10055,7 +10055,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3005</v>
+        <v>3015</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10321,7 +10321,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6076</v>
+        <v>6198.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10727,7 +10727,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12790</v>
+        <v>16440</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1031</v>
+        <v>1041</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11315,7 +11315,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3640</v>
+        <v>3715</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11595,7 +11595,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1482</v>
+        <v>1532</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11791,7 +11791,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>38336</v>
+        <v>39041</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12743,7 +12743,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13275,7 +13275,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3100</v>
+        <v>4835</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13597,7 +13597,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2500</v>
+        <v>2850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13695,7 +13695,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2275</v>
+        <v>2775</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13821,7 +13821,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1035</v>
+        <v>1045</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13989,7 +13989,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5100</v>
+        <v>5300</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14339,7 +14339,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>408.32</v>
+        <v>658.3199999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15106,7 +15106,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mallory aaren cook</t>
+          <t>timothy towne</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15119,11 +15119,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15134,7 +15134,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>timothy towne</t>
+          <t>mallory aaren cook</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15147,7 +15147,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -15893,7 +15893,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1095.54</v>
+        <v>1115.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16044,7 +16044,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>roland daniel martin</t>
+          <t>roger clarence albert</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -16057,11 +16057,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16072,7 +16072,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>roger clarence albert</t>
+          <t>roland daniel martin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -16085,11 +16085,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16999,7 +16999,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17377,7 +17377,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3050</v>
+        <v>4550</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17601,7 +17601,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>510</v>
+        <v>625</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17769,7 +17769,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11506.76</v>
+        <v>11526.76</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17867,7 +17867,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>2100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19099,7 +19099,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2575</v>
+        <v>2625</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19225,7 +19225,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8019.8</v>
+        <v>8319.799999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19351,7 +19351,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16740</v>
+        <v>18040</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19379,7 +19379,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2705.18</v>
+        <v>3756.18</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Weekly data update July 27: 315 new state transactions, fresh scraper run
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>778029.76</v>
+        <v>792720.92</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>337118</v>
+        <v>337168</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9509,7 +9509,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>8330</v>
+        <v>10405</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14087,7 +14087,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5925</v>
+        <v>6775</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17027,7 +17027,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>110</v>
+        <v>310</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17965,7 +17965,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3500</v>
+        <v>3630.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18259,7 +18259,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15250</v>
+        <v>15275</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19099,7 +19099,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2625</v>
+        <v>2870</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Use filing summary totals for governor candidates, add methodology footnote
Governor contribution/expenditure totals now based on Maine Ethics Commission
filing summaries (includes unitemized contributions and loans). R script adds
incremental transactions between filing periods. Footnote added to governor page.
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2432116.4</v>
+        <v>3039523.78</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nirav shah</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -660,11 +660,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E5">
-        <v>1246868.85</v>
+        <v>1334066.66</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>angus s king iii</t>
+          <t>nirav shah</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1194028.86</v>
+        <v>1246868.85</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>troy dale jackson</t>
+          <t>angus s king iii</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>912130.76</v>
+        <v>1194028.86</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>troy dale jackson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -735,11 +735,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E8">
-        <v>792720.92</v>
+        <v>912130.76</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>688181.97</v>
+        <v>781017.95</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Filing overlay for all 453 state candidates, fix PAC contribution counting
Scrape filing summaries for all state candidates (Rep/Sen/Gov) with
resume capability and incremental writes. Fix overlay formula to add
PAC contributions separately (not included in filing totals). Add name
mapping bridge table for ~100 candidates whose filer URL names differ
from candidate list. Fix HTML entities in filer names.
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -575,7 +575,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>hannah pingree</t>
+          <t>jonathan bush</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -585,11 +585,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>3039523.78</v>
+        <v>3217769.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -600,7 +600,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>shenna bellows</t>
+          <t>hannah pingree</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1672883.28</v>
+        <v>3041723.78</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>jonathan bush</t>
+          <t>angus s king iii</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -635,11 +635,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>1447420</v>
+        <v>2065629.93</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>robert b charles</t>
+          <t>shenna bellows</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -660,11 +660,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E5">
-        <v>1334066.66</v>
+        <v>1914913.56</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1246868.85</v>
+        <v>1478574.28</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>angus s king iii</t>
+          <t>robert b charles</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -710,11 +710,11 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E7">
-        <v>1194028.86</v>
+        <v>1335066.66</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>troy dale jackson</t>
+          <t>benjamin midgley</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -735,11 +735,11 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E8">
-        <v>912130.76</v>
+        <v>1136899</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>richard bennett</t>
+          <t>troy dale jackson</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -760,11 +760,11 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E9">
-        <v>781017.95</v>
+        <v>1079415.73</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>david john jones</t>
+          <t>richard bennett</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -785,11 +785,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E10">
-        <v>499329.22</v>
+        <v>781022.95</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>owen mccarthy</t>
+          <t>david john jones</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>386477.21</v>
+        <v>553696.87</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>benjamin midgley</t>
+          <t>owen mccarthy</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>337168</v>
+        <v>541291.22</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         </is>
       </c>
       <c r="E13">
-        <v>175753.68</v>
+        <v>232302.82</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="E14">
-        <v>44638.19</v>
+        <v>63962.58</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>james libby</t>
+          <t>john michael glowa sr</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -910,11 +910,11 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E15">
-        <v>15259.7</v>
+        <v>29583.92</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>w edward crockett</t>
+          <t>derek allen levasseur</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="E16">
-        <v>8835</v>
+        <v>24847.78</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>kenneth a capron</t>
+          <t>james libby</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E17">
-        <v>3450</v>
+        <v>17389.7</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>derek allen levasseur</t>
+          <t>w edward crockett</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="E18">
-        <v>1150</v>
+        <v>9317.98</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>john michael glowa sr</t>
+          <t>kenneth a capron</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1010,11 +1010,11 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E19">
-        <v>1150</v>
+        <v>3316.87</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1137,7 +1137,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>990</v>
+        <v>993.59</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1333,7 +1333,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1000.66</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1361,7 +1361,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>820</v>
+        <v>920</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>3228.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2565</v>
+        <v>4805</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3300</v>
+        <v>9833.75</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1386.18</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1949,7 +1949,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7619.56</v>
+        <v>12371.1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3222.5</v>
+        <v>8222.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2212,7 +2212,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>melanie ann tompkins</t>
+          <t>donald james ardell</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2225,11 +2225,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>146.23</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2240,7 +2240,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>donald james ardell</t>
+          <t>melanie ann tompkins</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9175.120000000001</v>
+        <v>13301.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2621,7 +2621,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4700</v>
+        <v>8733.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>800</v>
+        <v>819</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>7550</v>
+        <v>14367.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2747,7 +2747,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>945</v>
+        <v>945.03</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3930</v>
+        <v>4050.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2845,7 +2845,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>523</v>
+        <v>423</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2860,7 +2860,7 @@
 
 <file path=xl/worksheets/sheet115.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -2915,7 +2915,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>850</v>
+        <v>900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2926,7 +2926,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>scott strom</t>
+          <t>jeremy r mcarthur</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2946,6 +2946,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_65</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>scott strom</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>65</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_65</t>
         </is>
@@ -3111,7 +3139,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1170</v>
+        <v>5106</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3139,7 +3167,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>1000.08</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3192,7 +3220,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>zachary lejonhud</t>
+          <t>amanda noelle collamore</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3205,11 +3233,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1006</v>
+        <v>5022.09</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3220,7 +3248,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>amanda noelle collamore</t>
+          <t>zachary lejonhud</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3233,11 +3261,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1001</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3307,7 +3335,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>650</v>
+        <v>2410.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3335,7 +3363,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>500</v>
+        <v>2198.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3405,7 +3433,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>10100</v>
+        <v>11200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3433,7 +3461,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>950</v>
+        <v>961</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3486,7 +3514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>matthew rush</t>
+          <t>jantzen stephen craine</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3499,11 +3527,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>2070</v>
+        <v>4408.48</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3514,7 +3542,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jantzen stephen craine</t>
+          <t>matthew rush</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3527,11 +3555,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>981.15</v>
+        <v>2070</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3601,7 +3629,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1500</v>
+        <v>3134.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3699,7 +3727,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6685</v>
+        <v>8141.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3825,7 +3853,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>900</v>
+        <v>919.47</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3895,7 +3923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4425</v>
+        <v>5475</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4004,7 +4032,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>russell john black</t>
+          <t>marc edwards</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4017,11 +4045,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1480</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4032,7 +4060,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>marc edwards</t>
+          <t>russell john black</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4045,11 +4073,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>380</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4119,7 +4147,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15070</v>
+        <v>26355.95</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4147,7 +4175,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2000</v>
+        <v>7900</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4343,7 +4371,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>115</v>
+        <v>580</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4469,7 +4497,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2350</v>
+        <v>3574.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4497,7 +4525,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4567,7 +4595,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6025</v>
+        <v>9136.700000000001</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4595,7 +4623,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>880</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4665,7 +4693,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>750</v>
+        <v>1250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4693,7 +4721,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>170</v>
+        <v>1120</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4763,7 +4791,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1200</v>
+        <v>2450</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4833,7 +4861,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2200</v>
+        <v>4720</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4844,7 +4872,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>azalea cormier</t>
+          <t>gino valeriani</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4857,11 +4885,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1020</v>
+        <v>1995</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4872,7 +4900,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>gino valeriani</t>
+          <t>azalea cormier</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4885,11 +4913,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
-        <v>750</v>
+        <v>1020</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -4942,7 +4970,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>christopher easton</t>
+          <t>peter conley wood</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4955,11 +4983,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>4551.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4970,7 +4998,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>peter conley wood</t>
+          <t>christopher easton</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4983,11 +5011,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>350</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5057,7 +5085,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>925</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5085,7 +5113,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5155,7 +5183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2080</v>
+        <v>2434.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5183,7 +5211,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>1015</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5253,7 +5281,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>675</v>
+        <v>1025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5281,7 +5309,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5351,7 +5379,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2213.65</v>
+        <v>3008.65</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5362,7 +5390,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>paul welch</t>
+          <t>adrienne paul</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5375,11 +5403,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>850</v>
+        <v>1412</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5390,7 +5418,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>adrienne paul</t>
+          <t>paul welch</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5403,11 +5431,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>612</v>
+        <v>860</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5477,7 +5505,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2821.89</v>
+        <v>4389.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5505,7 +5533,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>945</v>
+        <v>990</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5575,7 +5603,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6783.7</v>
+        <v>16204.77</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5673,7 +5701,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>160</v>
+        <v>310</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5701,7 +5729,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>0.87</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5771,7 +5799,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3091.7</v>
+        <v>6155.59</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5799,7 +5827,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1110</v>
+        <v>1250</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5869,7 +5897,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12760</v>
+        <v>18411.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5950,7 +5978,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nicole richards</t>
+          <t>arthur k mingo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5963,11 +5991,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>2705.29</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5978,7 +6006,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>arthur k mingo</t>
+          <t>nicole richards</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5991,7 +6019,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -6065,7 +6093,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>73158.3</v>
+        <v>143087.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6093,7 +6121,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>700</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6121,7 +6149,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>305</v>
+        <v>325.04</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -6191,7 +6219,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1201.53</v>
+        <v>8155.22</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6272,7 +6300,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>scott girardin</t>
+          <t>stephen j wood</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6285,11 +6313,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6300,7 +6328,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>stephen j wood</t>
+          <t>scott girardin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6313,7 +6341,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
@@ -6332,7 +6360,7 @@
 
 <file path=xl/worksheets/sheet146.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -6370,7 +6398,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>julia a g mccabe</t>
+          <t>chad syphers</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6383,11 +6411,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1170</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6398,7 +6426,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chad syphers</t>
+          <t>julia a g mccabe</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6411,13 +6439,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>970</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_93</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>susan g longchamps</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>93</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Republican</t>
         </is>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_93</t>
         </is>
@@ -6468,7 +6524,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>janet beaudoin</t>
+          <t>scott a harriman</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6481,11 +6537,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>3850</v>
+        <v>33390.33</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6496,7 +6552,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>scott a harriman</t>
+          <t>janet beaudoin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6509,11 +6565,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>11203.6</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6583,7 +6639,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8201</v>
+        <v>56622.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6594,7 +6650,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>matthew kershaw</t>
+          <t>bret michael martel</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6607,11 +6663,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>927.53</v>
+        <v>2551.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6622,7 +6678,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bret michael martel</t>
+          <t>matthew kershaw</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -6635,11 +6691,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1768.82</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -6692,7 +6748,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>kerryl lee clement</t>
+          <t>luke jensen</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6705,11 +6761,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1085</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6720,7 +6776,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>luke jensen</t>
+          <t>kerryl lee clement</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6733,11 +6789,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>85</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6807,7 +6863,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1600</v>
+        <v>2550</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7059,7 +7115,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>500</v>
+        <v>686</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -7255,7 +7311,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1634</v>
+        <v>1634.8</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7270,7 +7326,7 @@
 
 <file path=xl/worksheets/sheet154.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -7356,6 +7412,34 @@
         <v>551</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jaric t fontaine</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>10</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Senator_10</t>
         </is>
@@ -7406,7 +7490,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>glenn chip curry</t>
+          <t>ryan christopher otis</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7419,11 +7503,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>3045</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7434,7 +7518,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ryan christopher otis</t>
+          <t>glenn chip curry</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7447,11 +7531,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>3000</v>
+        <v>2940</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7521,7 +7605,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1500</v>
+        <v>4500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7745,7 +7829,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5000</v>
+        <v>17727.06</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7773,7 +7857,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>4733.34</v>
+        <v>13069.13</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7843,7 +7927,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3105</v>
+        <v>3075</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7871,7 +7955,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1300</v>
+        <v>1490</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8039,7 +8123,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2905</v>
+        <v>2906</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8109,7 +8193,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2225.5</v>
+        <v>3858.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8120,7 +8204,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jojean keller</t>
+          <t>joshua morris</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8133,11 +8217,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1350</v>
+        <v>3089.39</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8148,7 +8232,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>joshua morris</t>
+          <t>jojean keller</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8161,11 +8245,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1416</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8235,7 +8319,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9604.48</v>
+        <v>12217.32</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8263,7 +8347,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2965</v>
+        <v>2865</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8333,7 +8417,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4100</v>
+        <v>7299</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8344,7 +8428,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>peter j southam</t>
+          <t>david duguay</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8357,11 +8441,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>2835</v>
+        <v>5100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8372,7 +8456,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>david duguay</t>
+          <t>peter j southam</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8385,11 +8469,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>2835</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8404,7 +8488,7 @@
 
 <file path=xl/worksheets/sheet164.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -8442,7 +8526,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>harold hull</t>
+          <t>harold trey l iii stewart</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8455,11 +8539,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>50</v>
+        <v>2495</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8470,7 +8554,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>harold trey l iii stewart</t>
+          <t>harold hull</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8483,13 +8567,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
+        <v>50</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>janel c underwoodcharette</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Senator_2</t>
         </is>
@@ -8557,7 +8669,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2935</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8585,7 +8697,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2885</v>
+        <v>3000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8655,7 +8767,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>19730</v>
+        <v>29319.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8683,7 +8795,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2463</v>
+        <v>3000.99</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8781,7 +8893,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2994.2</v>
+        <v>3029.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8879,7 +8991,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>2723.1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8907,7 +9019,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>700</v>
+        <v>2395</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8977,7 +9089,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5775</v>
+        <v>6000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9145,7 +9257,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3400</v>
+        <v>3650</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9215,7 +9327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12000</v>
+        <v>40100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9271,7 +9383,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>2975</v>
+        <v>2885</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9341,7 +9453,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1400</v>
+        <v>1840</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9411,7 +9523,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1618.9</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9481,7 +9593,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>17000</v>
+        <v>24200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9509,7 +9621,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>10405</v>
+        <v>10593.17</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9524,7 +9636,7 @@
 
 <file path=xl/worksheets/sheet175.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -9579,7 +9691,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>12406.51</v>
+        <v>17863.07</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9607,7 +9719,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3000</v>
+        <v>6760.65</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9618,7 +9730,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>stanley short jr</t>
+          <t>ester franklin</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9635,9 +9747,37 @@
         </is>
       </c>
       <c r="E4">
+        <v>170</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Senator_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>stanley short jr</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E5">
         <v>0</v>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Senator_3</t>
         </is>
@@ -9650,7 +9790,7 @@
 
 <file path=xl/worksheets/sheet176.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -9705,7 +9845,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3425</v>
+        <v>3005</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9744,7 +9884,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>harry white</t>
+          <t>m thad moody</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -9764,6 +9904,34 @@
         <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>Senator_30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>harry white</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Senator_30</t>
         </is>
@@ -9776,7 +9944,7 @@
 
 <file path=xl/worksheets/sheet177.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -9842,7 +10010,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>garrett plummer</t>
+          <t>scott benedetto eccleston</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9862,6 +10030,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Senator_31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>garrett plummer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Senator</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>31</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Senator_31</t>
         </is>
@@ -9912,7 +10108,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>henry l ingwersen</t>
+          <t>jason g litalien</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9925,11 +10121,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E2">
-        <v>2400</v>
+        <v>5910.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9940,7 +10136,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jason g litalien</t>
+          <t>henry l ingwersen</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9953,11 +10149,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>1100</v>
+        <v>2950</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10027,7 +10223,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6425</v>
+        <v>22430.52</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10055,7 +10251,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3015</v>
+        <v>2960</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10251,7 +10447,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3044</v>
+        <v>3000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10349,7 +10545,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3101</v>
+        <v>3186</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10430,7 +10626,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>joseph paul guerin</t>
+          <t>chad richard perkins</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10447,7 +10643,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6120</v>
+        <v>8524.84</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10458,7 +10654,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>chad richard perkins</t>
+          <t>joseph paul guerin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10475,7 +10671,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>5974.7</v>
+        <v>6225</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10503,7 +10699,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>2250</v>
+        <v>4050</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10531,7 +10727,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>1540</v>
+        <v>1657</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -10559,7 +10755,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>20.18</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -10657,7 +10853,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1335</v>
+        <v>1340</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10727,7 +10923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16440</v>
+        <v>25620</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10783,7 +10979,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>925</v>
+        <v>950</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -10881,7 +11077,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1800</v>
+        <v>1825</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10934,7 +11130,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>leo christopher kenney</t>
+          <t>michael tipping</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -10947,11 +11143,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>2980</v>
+        <v>3100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10962,7 +11158,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>michael tipping</t>
+          <t>leo christopher kenney</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -10975,11 +11171,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>2400</v>
+        <v>2980</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11049,7 +11245,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3100</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11147,7 +11343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1041</v>
+        <v>1146</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11162,7 +11358,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -11217,7 +11413,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>26685.78</v>
+        <v>28352.13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11228,7 +11424,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>dana marie appleby</t>
+          <t>jennifer l levesque</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -11248,6 +11444,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dana marie appleby</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_1</t>
         </is>
@@ -11315,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3715</v>
+        <v>3940</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11455,7 +11679,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>750</v>
+        <v>3645</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11623,7 +11847,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11693,7 +11917,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>1600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11791,7 +12015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>39041</v>
+        <v>39562.31</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11834,7 +12058,7 @@
 
 <file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -11900,7 +12124,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>meagan smith</t>
+          <t>lucy louisa perkins</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -11913,13 +12137,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_121</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>meagan smith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>121</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_121</t>
         </is>
@@ -11987,7 +12239,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>3968.42</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12155,7 +12407,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>400</v>
+        <v>4865.4</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12166,7 +12418,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>william r tuell</t>
+          <t>genevieve lemire</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -12179,11 +12431,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>400</v>
+        <v>690</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12194,7 +12446,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>genevieve lemire</t>
+          <t>william r tuell</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -12207,11 +12459,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E4">
-        <v>175</v>
+        <v>400</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -12309,7 +12561,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>985</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12477,7 +12729,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4325</v>
+        <v>6441.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12505,7 +12757,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2100</v>
+        <v>3226.31</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12743,7 +12995,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>360</v>
+        <v>5761.24</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12911,7 +13163,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>900</v>
+        <v>977.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12939,7 +13191,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>300</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13107,7 +13359,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>140</v>
+        <v>1334.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13177,7 +13429,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13275,7 +13527,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4835</v>
+        <v>11166.16</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13373,7 +13625,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3600</v>
+        <v>3676</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13471,7 +13723,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>980</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13499,7 +13751,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>947</v>
+        <v>947.02</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13597,7 +13849,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2850</v>
+        <v>6700</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13695,7 +13947,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2775</v>
+        <v>11258.71</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13723,7 +13975,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>945</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13793,7 +14045,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2500</v>
+        <v>5900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13821,7 +14073,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1045</v>
+        <v>1095</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -13891,7 +14143,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2555</v>
+        <v>2975</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14087,7 +14339,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6775</v>
+        <v>21819.2</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14115,7 +14367,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14185,7 +14437,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2472.72</v>
+        <v>7084.73</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14213,7 +14465,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>1000.98</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14269,7 +14521,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>775</v>
+        <v>1000</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -14367,7 +14619,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14382,7 +14634,7 @@
 
 <file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14448,7 +14700,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>gordon frohloff</t>
+          <t>domingo e torres</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14468,6 +14720,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_142</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>gordon frohloff</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>142</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_142</t>
         </is>
@@ -14480,7 +14760,7 @@
 
 <file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14535,7 +14815,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2000</v>
+        <v>3000.04</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14566,6 +14846,34 @@
         <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_143</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>melissa a simpson</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>143</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Republican</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_143</t>
         </is>
@@ -14578,7 +14886,7 @@
 
 <file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14616,7 +14924,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>corinna cole</t>
+          <t>jeff adams</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14629,11 +14937,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>371.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14644,7 +14952,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jeff adams</t>
+          <t>corinna cole</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14657,13 +14965,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E3">
+        <v>50</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_144</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>karen a gerrish</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>144</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Republican</t>
         </is>
       </c>
-      <c r="E3">
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_144</t>
         </is>
@@ -14759,7 +15095,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>950</v>
+        <v>995</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14942,7 +15278,7 @@
 
 <file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -14997,7 +15333,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>3509.36</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15036,7 +15372,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>noah cobb</t>
+          <t>marissa l tasker</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -15049,13 +15385,41 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
+        <is>
+          <t>Representative_148</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>noah cobb</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>148</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Unenrolled</t>
+        </is>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>Representative_148</t>
         </is>
@@ -15123,7 +15487,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1100</v>
+        <v>3400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15330,7 +15694,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>mark frederick zimmer</t>
+          <t>alexandros orestis</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15343,11 +15707,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>920</v>
+        <v>1075</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15358,7 +15722,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>alexandros orestis</t>
+          <t>mark frederick zimmer</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -15371,11 +15735,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>875</v>
+        <v>920</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -15445,7 +15809,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1450</v>
+        <v>3229.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15543,7 +15907,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>200</v>
+        <v>1600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15767,7 +16131,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>13010</v>
+        <v>15929.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15963,7 +16327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>8232.709999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15991,7 +16355,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16061,7 +16425,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1500</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16187,7 +16551,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16313,7 +16677,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>100</v>
+        <v>138.22</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -16383,7 +16747,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>750</v>
+        <v>1299.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16565,7 +16929,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>700</v>
+        <v>725</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -16635,7 +16999,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>975</v>
+        <v>1175</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16705,7 +17069,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16999,7 +17363,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>850</v>
+        <v>5301.02</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17027,7 +17391,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>310</v>
+        <v>385</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17097,7 +17461,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1290</v>
+        <v>1290.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17195,7 +17559,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>985</v>
+        <v>1035</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17223,7 +17587,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>950</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17251,7 +17615,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>525</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17262,7 +17626,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nancy theriaultspecial</t>
+          <t>james michael michaud</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17279,7 +17643,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>964.33</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -17290,7 +17654,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>james michael michaud</t>
+          <t>nancy theriaultspecial</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -17377,7 +17741,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4550</v>
+        <v>6100</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17405,7 +17769,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>850</v>
+        <v>950</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17433,7 +17797,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>313.39</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17503,7 +17867,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>600</v>
+        <v>2784.51</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17584,7 +17948,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eric boothroyd</t>
+          <t>andrew r torbett</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17597,11 +17961,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>625</v>
+        <v>3565</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17612,7 +17976,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>andrew r torbett</t>
+          <t>eric boothroyd</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17625,11 +17989,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>500</v>
+        <v>1125</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17699,7 +18063,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>500</v>
+        <v>2950</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17769,7 +18133,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>11526.76</v>
+        <v>12731.79</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17797,7 +18161,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>900</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17867,7 +18231,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2100</v>
+        <v>2600.66</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17895,7 +18259,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>42.54</v>
+        <v>168.54</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17965,7 +18329,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3630.65</v>
+        <v>18002.47</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18046,7 +18410,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>james e thorne</t>
+          <t>debora farnham</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18059,11 +18423,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>100</v>
+        <v>505</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18074,7 +18438,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>debora farnham</t>
+          <t>james e thorne</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18087,11 +18451,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18259,7 +18623,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>15275</v>
+        <v>33840.49</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18287,7 +18651,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>950</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18340,7 +18704,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>kayla miller</t>
+          <t>benjamin charles hymes</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -18353,11 +18717,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>900</v>
+        <v>2437.56</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18385,7 +18749,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>310</v>
+        <v>1210</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18396,7 +18760,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>benjamin charles hymes</t>
+          <t>kayla miller</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -18409,11 +18773,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
-        <v>300</v>
+        <v>900</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -18483,7 +18847,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2850</v>
+        <v>3850</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18651,7 +19015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1150</v>
+        <v>1210</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18749,7 +19113,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1070</v>
+        <v>3070</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -18973,7 +19337,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>555</v>
+        <v>1673.46</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19054,7 +19418,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>chris p austin</t>
+          <t>rhiannon hampson</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19067,11 +19431,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>4779.74</v>
+        <v>9604.469999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19082,7 +19446,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>rhiannon hampson</t>
+          <t>chris p austin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19095,11 +19459,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>2870</v>
+        <v>5335.5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19225,7 +19589,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8319.799999999999</v>
+        <v>8369.799999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19236,7 +19600,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>shawn saindon</t>
+          <t>brady alden clark</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19249,11 +19613,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E3">
-        <v>1013.84</v>
+        <v>2006.2</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19264,7 +19628,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>brady alden clark</t>
+          <t>shawn saindon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19277,11 +19641,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1063.84</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19351,7 +19715,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>18040</v>
+        <v>24962</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19379,7 +19743,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3756.18</v>
+        <v>5530.13</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19575,7 +19939,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>850</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19726,7 +20090,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nicolas john hamlin</t>
+          <t>trent vellella</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19739,11 +20103,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E2">
-        <v>1000</v>
+        <v>1025</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19754,7 +20118,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>suzanne r andresen</t>
+          <t>nicolas john hamlin</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19782,7 +20146,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>trent vellella</t>
+          <t>suzanne r andresen</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19795,11 +20159,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E4">
-        <v>925</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19814,7 +20178,7 @@
 
 <file path=xl/worksheets/sheet98.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -19880,7 +20244,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bruce archer</t>
+          <t>lori g kenneson</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19900,6 +20264,34 @@
         <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
+        <is>
+          <t>Representative_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>bruce archer</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Representative</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>5</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Democratic</t>
+        </is>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>Representative_5</t>
         </is>
@@ -19950,7 +20342,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>david a sinclair</t>
+          <t>jedediah j rice</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19963,11 +20355,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19978,7 +20370,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jedediah j rice</t>
+          <t>david a sinclair</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19991,7 +20383,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">

</xml_diff>

<commit_message>
Weekly update Aug 10: 3,688 new state transactions, fresh filing overlay
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -7633,7 +7633,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6198.57</v>
+        <v>6248.57</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12995,7 +12995,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5761.24</v>
+        <v>5786.24</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix double-counting: use filing totals directly, filter phantom expenditures
- Remove PAC and incremental additions from filing overlay (filing total is authoritative)
- Filter 39 phantom expenditures from carryover transfers
- Fix Roy Gott office (Senator, not Representative) in filer URLs
- Add name merge for roy d gott
- Updated MCEA filings, new transactions, clean output data
</commit_message>
<xml_diff>
--- a/viz/data/clean/maine_races_by_district.xlsx
+++ b/viz/data/clean/maine_races_by_district.xlsx
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3041723.78</v>
+        <v>3039523.78</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>1914913.56</v>
+        <v>1910163.56</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -689,7 +689,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>1478574.28</v>
+        <v>1476415.96</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -714,7 +714,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>1335066.66</v>
+        <v>1334066.66</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -739,7 +739,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>1136899</v>
+        <v>1133469</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E10">
-        <v>781022.95</v>
+        <v>781017.95</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="E11">
-        <v>553696.87</v>
+        <v>551996.87</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="E12">
-        <v>541291.22</v>
+        <v>539837.01</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
         </is>
       </c>
       <c r="E17">
-        <v>17389.7</v>
+        <v>17025</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1753,7 +1753,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1660</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8222.5</v>
+        <v>7892.5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1370</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1145</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>21.15</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2551,7 +2551,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>211</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>14367.43</v>
+        <v>12967.43</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1001</v>
+        <v>951</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2410.03</v>
+        <v>2210.03</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2070</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>8141.7</v>
+        <v>8116.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -3755,7 +3755,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3853,7 +3853,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>919.47</v>
+        <v>819.47</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5475</v>
+        <v>4975</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -4721,7 +4721,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1120</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -4917,7 +4917,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1020</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -5183,7 +5183,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2434.58</v>
+        <v>2254.58</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1025</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5407,7 +5407,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1412</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -5505,7 +5505,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4389.7</v>
+        <v>3464.7</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5603,7 +5603,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>16204.77</v>
+        <v>15721.07</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>310</v>
+        <v>250</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -5827,7 +5827,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1250</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6093,7 +6093,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>143087.25</v>
+        <v>142847.25</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6524,7 +6524,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>scott a harriman</t>
+          <t>janet beaudoin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6537,11 +6537,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>33390.33</v>
+        <v>11203.6</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6552,7 +6552,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>janet beaudoin</t>
+          <t>scott a harriman</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6565,11 +6565,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>11203.6</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -6695,7 +6695,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1768.82</v>
+        <v>1718.82</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>luke jensen</t>
+          <t>kerryl lee clement</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6761,11 +6761,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1085</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -6776,7 +6776,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kerryl lee clement</t>
+          <t>luke jensen</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
@@ -7283,7 +7283,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2555</v>
+        <v>2400</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -7409,7 +7409,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>551</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7616,7 +7616,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ann higgins matlack</t>
+          <t>roy gott</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7629,11 +7629,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Unenrolled</t>
         </is>
       </c>
       <c r="E3">
-        <v>300</v>
+        <v>100</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -7644,7 +7644,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>roy gott</t>
+          <t>ann higgins matlack</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Unenrolled</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">
@@ -7927,7 +7927,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3075</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2906</v>
+        <v>2736</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8249,7 +8249,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1416</v>
+        <v>1316</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -8767,7 +8767,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>29319.01</v>
+        <v>28964.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -8893,7 +8893,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3029.2</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9089,7 +9089,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6000</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9159,7 +9159,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>4075</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9257,7 +9257,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3650</v>
+        <v>3450</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9593,7 +9593,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>24200</v>
+        <v>23200</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9621,7 +9621,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>10593.17</v>
+        <v>193.17</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -9747,7 +9747,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -9845,7 +9845,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3005</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1100</v>
+        <v>900</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10251,7 +10251,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>2960</v>
+        <v>2795</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10419,7 +10419,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3055</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10517,7 +10517,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>6248.57</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -10545,7 +10545,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>3186</v>
+        <v>2885</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -10853,7 +10853,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1340</v>
+        <v>905</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -11147,7 +11147,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3100</v>
+        <v>3000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1146</v>
+        <v>871</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11413,7 +11413,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>28352.13</v>
+        <v>28102.13</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11539,7 +11539,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3940</v>
+        <v>3765</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11679,7 +11679,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3645</v>
+        <v>2895</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -11819,7 +11819,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1532</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12015,7 +12015,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>39562.31</v>
+        <v>38677.31</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12113,7 +12113,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12239,7 +12239,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>3968.42</v>
+        <v>3868.42</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12309,7 +12309,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12435,7 +12435,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>690</v>
+        <v>515</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -12533,7 +12533,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1060</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -12995,7 +12995,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5786.24</v>
+        <v>5411.24</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -13653,7 +13653,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1275</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14073,7 +14073,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1095</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14241,7 +14241,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>5300</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14269,7 +14269,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14574,7 +14574,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>poppy t arford</t>
+          <t>ravi jackson</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -14587,11 +14587,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>658.3199999999999</v>
+        <v>80</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -14602,7 +14602,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ravi jackson</t>
+          <t>poppy t arford</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -14615,11 +14615,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E3">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -14689,7 +14689,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1160</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -15711,7 +15711,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1075</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16257,7 +16257,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1115.54</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16845,7 +16845,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -16873,7 +16873,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1050</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -16884,7 +16884,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>joschka winterling</t>
+          <t>victoria porter kornfield</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -16901,7 +16901,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>792.27</v>
+        <v>725</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -16912,7 +16912,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>victoria porter kornfield</t>
+          <t>joschka winterling</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -16929,7 +16929,7 @@
         </is>
       </c>
       <c r="E5">
-        <v>725</v>
+        <v>452.27</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -16999,7 +16999,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1175</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17139,7 +17139,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>2555</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17391,7 +17391,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17461,7 +17461,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>1290.01</v>
+        <v>1000.01</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17542,7 +17542,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nancy mcdowell</t>
+          <t>nancy jean theriault</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -17555,11 +17555,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1035</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -17570,7 +17570,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nancy mcdowellspecial</t>
+          <t>nancy mcdowell</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -17587,7 +17587,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1000</v>
+        <v>975</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -17598,7 +17598,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nancy jean theriault</t>
+          <t>james michael michaud</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -17615,7 +17615,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1000</v>
+        <v>964.33</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -17626,7 +17626,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>james michael michaud</t>
+          <t>nancy mcdowellspecial</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -17639,11 +17639,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E5">
-        <v>964.33</v>
+        <v>950</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -17993,7 +17993,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1125</v>
+        <v>600</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18732,7 +18732,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>jason cherry</t>
+          <t>kayla miller</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -18749,7 +18749,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1210</v>
+        <v>900</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -18760,7 +18760,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>kayla miller</t>
+          <t>jason cherry</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19124,7 +19124,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>marcus mrowka</t>
+          <t>joshua d gerritsen</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19141,7 +19141,7 @@
         </is>
       </c>
       <c r="E3">
-        <v>1070</v>
+        <v>1000</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -19152,7 +19152,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>joshua d gerritsen</t>
+          <t>marcus mrowka</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -19169,7 +19169,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1000</v>
+        <v>970</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19435,7 +19435,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>9604.469999999999</v>
+        <v>9334.469999999999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -19645,7 +19645,7 @@
         </is>
       </c>
       <c r="E4">
-        <v>1063.84</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -19715,7 +19715,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>24962</v>
+        <v>24487</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -20090,7 +20090,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>trent vellella</t>
+          <t>nicolas john hamlin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20103,11 +20103,11 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Democratic</t>
+          <t>Republican</t>
         </is>
       </c>
       <c r="E2">
-        <v>1025</v>
+        <v>1000</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -20118,7 +20118,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nicolas john hamlin</t>
+          <t>suzanne r andresen</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -20146,7 +20146,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>suzanne r andresen</t>
+          <t>trent vellella</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -20159,7 +20159,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Republican</t>
+          <t>Democratic</t>
         </is>
       </c>
       <c r="E4">

</xml_diff>